<commit_message>
feat(import): templates list valid codes; import validates category and channel [G9-M24]
Templates never showed which property codes, channels or expense
categories were valid. Unknown categories fell silently into 'Diger' and
channels were stored as free text next to the form's codes. Now:
- templates carry step-by-step instructions and a valid-values sheet
  (the in-app one with the tenant's own codes); one guide module serves
  both the in-app and published templates
- import maps category/channel names to canonical values and rejects
  unknown ones with the valid list; values already in the ledger are
  accepted verbatim so export -> re-import still round-trips
- template example rows can no longer be imported as real data (the
  expense 'ALL' row and the in-app examples with real codes could)
- import screen shows valid values and a ChatGPT prompt that converts
  the user's own table into the template

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sablonlar/lexbnb-gider-sablonu.xlsx
+++ b/sablonlar/lexbnb-gider-sablonu.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Giderler" sheetId="1" r:id="rId1"/>
     <sheet name="NASIL DOLDURULUR" sheetId="2" r:id="rId2"/>
+    <sheet name="GEÇERLİ DEĞERLER" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -425,19 +426,19 @@
         <v>2026-07-03</v>
       </c>
       <c r="B2" t="str">
-        <v>Şömine &amp; Yakacak</v>
+        <v>Fatura</v>
       </c>
       <c r="C2" t="str">
         <v>18000</v>
       </c>
       <c r="D2" t="str">
-        <v>Örnek: yakacak alımı</v>
+        <v>Örnek: elektrik faturası</v>
       </c>
       <c r="E2" t="str">
         <v>OPEX</v>
       </c>
       <c r="F2" t="str">
-        <v>ALL</v>
+        <v>MULK_KODU_1</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +446,7 @@
         <v>2026-07-08</v>
       </c>
       <c r="B3" t="str">
-        <v>Bakım &amp; Onarım</v>
+        <v>Bakım</v>
       </c>
       <c r="C3" t="str">
         <v>6500</v>
@@ -465,7 +466,7 @@
         <v>2026-07-14</v>
       </c>
       <c r="B4" t="str">
-        <v>Yatırım &amp; Demirbaş</v>
+        <v>Diğer</v>
       </c>
       <c r="C4" t="str">
         <v>45000</v>
@@ -489,11 +490,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>LEXBNB — GİDER DEFTERİ ŞABLONU</v>
+        <v>LEXBNB — GİDER DEFTERİ ŞABLONU · NASIL DOLDURULUR</v>
       </c>
     </row>
     <row r="2">
@@ -503,77 +504,217 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ZORUNLU SÜTUNLAR: Tarih, Kategori, Tutar</v>
+        <v>ADIM 1 — İlk sayfadaki örnek satırları silin ya da üzerine yazın. Başlık satırı DOSYANIN İLK SATIRI olmalı.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Diğer sütunlar isteğe bağlıdır.</v>
+        <v>ADIM 2 — Her gider bir satırdır. ZORUNLU: Tarih, Kategori, Tutar.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>ADIM 3 — "Kategori": GEÇERLİ DEĞERLER sayfasındaki kategorilerden birini yazın (büyük/küçük harf önemsiz). Listede olmayan kategorinin satırı kaydedilmez ve nedeni yazılır — "Diğer"e sessizce düşmez.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>1) "Villa" sütunu boş veya ALL ise gider tüm portföye yazılır.</v>
+        <v>ADIM 4 — "Villa": boş ya da ALL ise gider tüm portföye yazılır. Tek mülke yazmak için kendi mülk kodunuzu girin; MULK_KODU_1 / MULK_KODU_2 yer tutucudur, değiştirmezseniz o satır kaydedilmez.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v xml:space="preserve">   Tek bir mülke yazmak için KENDİ mülk kodunuzu girin.</v>
+        <v>ADIM 5 — "Tür": OPEX (işletme gideri) ya da CAPEX (yatırım). Boşsa OPEX.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v xml:space="preserve">   MULK_KODU_1 / MULK_KODU_2 yalnızca yer tutucudur; değiştirmezseniz</v>
+        <v>ADIM 6 — Tarih: 2026-07-03 ya da 03.07.2026. Tutar: 18000 ya da 18.000,50.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v xml:space="preserve">   o satırlar kaydedilmez.</v>
+        <v>ADIM 7 — Temizlik personeline ödenen tutar buraya GİRİLMEZ; temizlik görevinden gider olarak yazılır. Reklam harcamasını Kanallar ve Pazarlama ekranından girin; burada da girilirse iki kez sayılır.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2) "Tür": OPEX (işletme gideri) veya CAPEX (yatırım). Boşsa OPEX sayılır.</v>
+        <v>ADIM 8 — Kaydedip Araçlar › Excel / CSV yükle ekranına bırakın. Önizlemede hatalı satırları ve nedenini görürsünüz; onaylamadan hiçbir şey kaydedilmez.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B23"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>KATEGORİLER — "Kategori" sütununa KATEGORİ adını yazın</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Neleri kapsar</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Maaş</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Maaş (Personel / Yönetici)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Temizlik</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Temizlik &amp; Çamaşırhane</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Bakım</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Bakım, Onarım &amp; Tesisat</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Reklam</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Reklam &amp; Pazarlama (Meta/Google)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Akaryakıt</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Akaryakıt &amp; Ulaşım</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Fatura</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Fatura (Elektrik, Su, İnternet)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Muhasebe</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Muhasebe &amp; Hukuk</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Kredi Kartı / Komisyon</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Kredi Kartı / Komisyon</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>3) Tarih: 2026-07-03 veya 03.07.2026 — ikisi de kabul edilir.</v>
+        <v>Danışmanlık</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Danışmanlık &amp; Yazılım</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>4) Tutar: 18000 veya 18.000,50 — ikisi de kabul edilir.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>5) Başlık satırı DOSYANIN İLK SATIRI olmalıdır.</v>
+        <v>Diğer</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Diğer Giderler</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>MÜLKLER — "Villa" sütunu (boş ya da ALL = tüm portföy)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>NOT: Temizlik personeline ödenen tutar buraya GİRİLMEZ; o, rezervasyonun</v>
+        <v>Kod</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Ad</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>temizlik görevinden otomatik gider yazılır.</v>
+        <v>ALL</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tüm portföy</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>MULK_KODU_1</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Yer tutucu — kendi mülk kodunuzu yazın. Kodlarınız hazır yazılı şablon için: uygulamada Araçlar › Excel / CSV yükle › "Kendi mülk kodlarınızla hazır şablon".</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>MULK_KODU_2</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Yer tutucu — kendi mülk kodunuzu yazın. Kodlarınız hazır yazılı şablon için: uygulamada Araçlar › Excel / CSV yükle › "Kendi mülk kodlarınızla hazır şablon".</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TÜR — "Tür" sütunu</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Değer</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Anlamı</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="B22" t="str">
+        <v>İşletme gideri (boşsa bu sayılır)</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>CAPEX</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Yatırım / demirbaş</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>